<commit_message>
Update result using cutoff threshold at 75th percentile
</commit_message>
<xml_diff>
--- a/result/icd9_inclusion_mapping_summary_LavenDist.xlsx
+++ b/result/icd9_inclusion_mapping_summary_LavenDist.xlsx
@@ -451,12 +451,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="75" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="75" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -485,220 +485,836 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1756</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Atherectomy of other non-coronary vessel(s)</t>
+          <t>Operations on other endocrine glands</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Directional atherectomy</t>
+          <t>operations on: pineal gland</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1753, 1754, 1755</t>
+          <t>0759</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1756</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Atherectomy of other non-coronary vessel(s)</t>
+          <t>Operations on other endocrine glands</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Excimer laser atherectomy</t>
+          <t>operations on: pituitary gland</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1753, 1754, 1755</t>
+          <t>0779</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1756</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Atherectomy of other non-coronary vessel(s)</t>
+          <t>Operations on other endocrine glands</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Rotational atherectomy</t>
+          <t>operations on: thymus</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1753, 1754, 1755</t>
+          <t>0141, 0799</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2096</t>
+          <t>143</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Implantation or replacement of cochlear prosthetic device, not otherwise specified</t>
+          <t>Repair of retinal tear</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>mastoidectomy</t>
+          <t>repair of retinal defect</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>3570</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2097</t>
+          <t>1756</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Implantation or replacement of cochlear prosthetic device, single channel</t>
+          <t>Atherectomy of other non-coronary vessel(s)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>mastoidectomy</t>
+          <t>Directional atherectomy</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>1753, 1755, 1754</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2098</t>
+          <t>1756</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Implantation or replacement of cochlear prosthetic device, multiple channel</t>
+          <t>Atherectomy of other non-coronary vessel(s)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>mastoidectomy</t>
+          <t>Excimer laser atherectomy</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>1753, 1755, 1754</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3897</t>
+          <t>1756</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Central venous catheter placement with guidance</t>
+          <t>Atherectomy of other non-coronary vessel(s)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>electrocardiogram</t>
+          <t>Rotational atherectomy</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>8952</t>
+          <t>1753, 1755, 1754</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>485</t>
+          <t>2096</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abdominoperineal resection of rectum</t>
+          <t>Implantation or replacement of cochlear prosthetic device, not otherwise specified</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Complete proctectomy</t>
+          <t>mastoidectomy</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2632</t>
+          <t>2021, 204, 854</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>727</t>
+          <t>2097</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Vacuum extraction</t>
+          <t>Implantation or replacement of cochlear prosthetic device, single channel</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Malström's extraction</t>
+          <t>mastoidectomy</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>7279</t>
+          <t>2021, 204, 854</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>2098</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Implantation or replacement of cochlear prosthetic device, multiple channel</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>mastoidectomy</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2021, 204, 854</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Operations on salivary glands and ducts</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>operations on: submaxillary gland and duct</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2699</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Other operations on mouth and face</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>operations on: lips</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>13, 08, 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Other operations on mouth and face</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>operations on: palate</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2799</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Operations on pharynx</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>operations on: hypopharynx</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2999</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Operations on pharynx</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>operations on: nasopharynx</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2999</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Operations on pharynx</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>operations on: oropharynx</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2999</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Operations on pharynx</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>operations on: pyriform sinus</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2999</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>3897</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Central venous catheter placement with guidance</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>electrocardiogram</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>8952</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>485</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Abdominoperineal resection of rectum</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Complete proctectomy</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2632</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Operations on gallbladder and biliary tract</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>operations on: sphincter of Oddi</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>5189</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Other operations on abdominal region</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>operations on: flank</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>49, 13</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Other operations on abdominal region</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>operations on: mesentery</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>5499</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Other operations on abdominal region</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>operations on: omentum</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>5499</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Other operations on abdominal region</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>operations on: peritoneum</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>5499</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Operations on urethra</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>operations on: periurethral tissue</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>5899, 4899</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>662</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Bilateral endoscopic destruction or occlusion of fallopian tubes</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>bilateral endoscopic destruction or occlusion of fallopian tubes by: culdoscopy</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>6629</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>662</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Bilateral endoscopic destruction or occlusion of fallopian tubes</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>bilateral endoscopic destruction or occlusion of fallopian tubes by: endoscopy</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>6629</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>662</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Bilateral endoscopic destruction or occlusion of fallopian tubes</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>bilateral endoscopic destruction or occlusion of fallopian tubes by: laparoscopy</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>6629</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>662</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Bilateral endoscopic destruction or occlusion of fallopian tubes</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>bilateral endoscopic destruction or occlusion of fallopian tubes by: peritoneoscopy</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>6629</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>727</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Vacuum extraction</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Malström's extraction</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>7279</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Incision and excision of joint structures</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>operations on: condyle</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Incision and excision of joint structures</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>operations on: ligament</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>8199</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>8053</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>Repair of the anulus fibrosus with graft or prosthesis</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>microsurgical suture repair with fascial autograft</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>8054</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Operations on skin and subcutaneous tissue</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>operations on: male perineum</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>718</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Operations on skin and subcutaneous tissue</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>operations on: nails</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>49, 13, 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>887</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Diagnostic ultrasound</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Non-invasive ultrasound</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>8872</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>887</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Diagnostic ultrasound</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Ultrasonography</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>9513, 8873</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>967</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Other continuous invasive mechanical ventilation</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Endotracheal respiratory assistance</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>3961</t>
         </is>
       </c>
     </row>

</xml_diff>